<commit_message>
chore: daily sync bitacora
</commit_message>
<xml_diff>
--- a/data/bitacora.xlsx
+++ b/data/bitacora.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupokaufmann-my.sharepoint.com/personal/samuel_sanchez_grupokaufmann_com/Documents/Documentos/Dev/bitacora_diaria/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="335" documentId="8_{4616FF0F-C10E-4DFE-8F27-869B9C60E0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7ACB77ED-ACC9-43BA-A194-CDEBA9184811}"/>
+  <xr:revisionPtr revIDLastSave="344" documentId="8_{4616FF0F-C10E-4DFE-8F27-869B9C60E0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E977F3E9-7E0D-4C1E-A20A-8DCF42B2E71A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A9E3F017-9040-47A2-B586-0486128F3261}"/>
   </bookViews>
@@ -1641,17 +1641,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{40364ABC-409D-4532-8E14-9D155F80C509}" name="Tabla1" displayName="Tabla1" ref="A1:J205" totalsRowShown="0">
-  <autoFilter ref="A1:J205" xr:uid="{40364ABC-409D-4532-8E14-9D155F80C509}">
-    <filterColumn colId="4">
-      <filters blank="1">
-        <filter val="ALEJANDRO ALBERTO VILLAGRA ORÓSTEGUI"/>
-        <filter val="ARTURO ANDRÉS SILVA ESPERGUE"/>
-        <filter val="BORIS ISRAEL CRUCES MARTÍNEZ"/>
-        <filter val="RODRIGO ANDRÉS INZUNZA LABRA"/>
-        <filter val="SERGIO ALBERTO ORELLANA VEGA"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:J205" xr:uid="{40364ABC-409D-4532-8E14-9D155F80C509}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{0A7C6585-5C8B-46BF-ABA0-2DA806D161DC}" name="FLOTA" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{EB7792BB-219D-496F-9F16-84F6805E0CB0}" name="VIN CON PROBLEMAS" dataDxfId="8"/>
@@ -2032,7 +2022,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="14.45" hidden="1">
+    <row r="2" spans="1:12" ht="14.45">
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
@@ -2055,7 +2045,7 @@
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
     </row>
-    <row r="3" spans="1:12" ht="14.45" hidden="1">
+    <row r="3" spans="1:12" ht="14.45">
       <c r="A3" s="7" t="s">
         <v>10</v>
       </c>
@@ -2078,7 +2068,7 @@
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
     </row>
-    <row r="4" spans="1:12" ht="14.45" hidden="1">
+    <row r="4" spans="1:12" ht="14.45">
       <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
@@ -2101,7 +2091,7 @@
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
     </row>
-    <row r="5" spans="1:12" ht="14.45" hidden="1">
+    <row r="5" spans="1:12" ht="14.45">
       <c r="A5" s="7" t="s">
         <v>10</v>
       </c>
@@ -2124,7 +2114,7 @@
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
     </row>
-    <row r="6" spans="1:12" ht="14.45" hidden="1">
+    <row r="6" spans="1:12" ht="14.45">
       <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
@@ -2147,7 +2137,7 @@
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
     </row>
-    <row r="7" spans="1:12" ht="14.45" hidden="1">
+    <row r="7" spans="1:12" ht="14.45">
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
@@ -2170,7 +2160,7 @@
       <c r="H7" s="24"/>
       <c r="I7" s="24"/>
     </row>
-    <row r="8" spans="1:12" ht="14.45" hidden="1">
+    <row r="8" spans="1:12" ht="14.45">
       <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
@@ -2193,7 +2183,7 @@
       <c r="H8" s="24"/>
       <c r="I8" s="24"/>
     </row>
-    <row r="9" spans="1:12" ht="14.45" hidden="1">
+    <row r="9" spans="1:12" ht="14.45">
       <c r="A9" s="7" t="s">
         <v>10</v>
       </c>
@@ -2216,7 +2206,7 @@
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
     </row>
-    <row r="10" spans="1:12" ht="14.45" hidden="1">
+    <row r="10" spans="1:12" ht="14.45">
       <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
@@ -2239,7 +2229,7 @@
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
     </row>
-    <row r="11" spans="1:12" ht="14.45" hidden="1">
+    <row r="11" spans="1:12" ht="14.45">
       <c r="A11" s="7" t="s">
         <v>10</v>
       </c>
@@ -2683,7 +2673,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="14.45" hidden="1">
+    <row r="30" spans="1:9" ht="14.45">
       <c r="A30" s="7" t="s">
         <v>80</v>
       </c>
@@ -2706,7 +2696,7 @@
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
     </row>
-    <row r="31" spans="1:9" ht="14.45" hidden="1">
+    <row r="31" spans="1:9" ht="14.45">
       <c r="A31" s="7" t="s">
         <v>80</v>
       </c>
@@ -2729,7 +2719,7 @@
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
     </row>
-    <row r="32" spans="1:9" ht="14.45" hidden="1">
+    <row r="32" spans="1:9" ht="14.45">
       <c r="A32" s="7" t="s">
         <v>80</v>
       </c>
@@ -2752,7 +2742,7 @@
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
     </row>
-    <row r="33" spans="1:9" ht="14.45" hidden="1">
+    <row r="33" spans="1:9" ht="14.45">
       <c r="A33" s="7" t="s">
         <v>80</v>
       </c>
@@ -2775,7 +2765,7 @@
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
     </row>
-    <row r="34" spans="1:9" ht="14.45" hidden="1">
+    <row r="34" spans="1:9" ht="14.45">
       <c r="A34" s="7" t="s">
         <v>80</v>
       </c>
@@ -2798,7 +2788,7 @@
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
     </row>
-    <row r="35" spans="1:9" ht="14.45" hidden="1">
+    <row r="35" spans="1:9" ht="14.45">
       <c r="A35" s="7" t="s">
         <v>80</v>
       </c>
@@ -2821,7 +2811,7 @@
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
     </row>
-    <row r="36" spans="1:9" ht="14.45" hidden="1">
+    <row r="36" spans="1:9" ht="14.45">
       <c r="A36" s="7" t="s">
         <v>80</v>
       </c>
@@ -3768,7 +3758,7 @@
       <c r="H72" s="12"/>
       <c r="I72" s="12"/>
     </row>
-    <row r="73" spans="1:9" ht="14.45" hidden="1">
+    <row r="73" spans="1:9" ht="14.45">
       <c r="A73" s="7" t="s">
         <v>172</v>
       </c>
@@ -3791,7 +3781,7 @@
       <c r="H73" s="12"/>
       <c r="I73" s="12"/>
     </row>
-    <row r="74" spans="1:9" ht="14.45" hidden="1">
+    <row r="74" spans="1:9" ht="14.45">
       <c r="A74" s="7" t="s">
         <v>172</v>
       </c>
@@ -4182,7 +4172,7 @@
       <c r="H90" s="12"/>
       <c r="I90" s="12"/>
     </row>
-    <row r="91" spans="1:9" ht="14.45" hidden="1">
+    <row r="91" spans="1:9" ht="14.45">
       <c r="A91" s="7" t="s">
         <v>210</v>
       </c>
@@ -4205,7 +4195,7 @@
       <c r="H91" s="12"/>
       <c r="I91" s="12"/>
     </row>
-    <row r="92" spans="1:9" ht="14.45" hidden="1">
+    <row r="92" spans="1:9" ht="14.45">
       <c r="A92" s="7" t="s">
         <v>210</v>
       </c>
@@ -4228,7 +4218,7 @@
       <c r="H92" s="12"/>
       <c r="I92" s="12"/>
     </row>
-    <row r="93" spans="1:9" ht="14.45" hidden="1">
+    <row r="93" spans="1:9" ht="14.45">
       <c r="A93" s="7" t="s">
         <v>210</v>
       </c>
@@ -4956,7 +4946,7 @@
       <c r="H123" s="12"/>
       <c r="I123" s="12"/>
     </row>
-    <row r="124" spans="1:9" ht="14.45" hidden="1">
+    <row r="124" spans="1:9" ht="14.45">
       <c r="A124" s="7" t="s">
         <v>287</v>
       </c>
@@ -4979,7 +4969,7 @@
       <c r="H124" s="12"/>
       <c r="I124" s="12"/>
     </row>
-    <row r="125" spans="1:9" ht="14.45" hidden="1">
+    <row r="125" spans="1:9" ht="14.45">
       <c r="A125" s="7" t="s">
         <v>287</v>
       </c>
@@ -5002,7 +4992,7 @@
       <c r="H125" s="12"/>
       <c r="I125" s="12"/>
     </row>
-    <row r="126" spans="1:9" ht="14.45" hidden="1">
+    <row r="126" spans="1:9" ht="14.45">
       <c r="A126" s="7" t="s">
         <v>287</v>
       </c>
@@ -6576,6 +6566,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100027709BF533FA442AFC4A8B2C0110727" ma:contentTypeVersion="15" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a37fc0d7c302f7619d355a49e1f175a4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="3e53c16e-6636-411e-b1c4-e9eeb71b3b2a" xmlns:ns4="bda9c1ec-c4e2-44f9-929c-ca399fe36c88" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="01250a30c504a808427f15ccf149ee4d" ns3:_="" ns4:_="">
     <xsd:import namespace="3e53c16e-6636-411e-b1c4-e9eeb71b3b2a"/>
@@ -6808,7 +6807,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_activity xmlns="3e53c16e-6636-411e-b1c4-e9eeb71b3b2a" xsi:nil="true"/>
@@ -6816,23 +6815,14 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C8123E5-81FD-4C24-91F1-33BC079967E9}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4794C7E6-B89D-4081-9A67-B8D500EF1EE4}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9861A25-610F-425F-BC6A-AC52D4971411}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C8123E5-81FD-4C24-91F1-33BC079967E9}"/>
 </file>
</xml_diff>